<commit_message>
Orden de eliminación de archivos y modificación de otros en el proyecto, incluyendo la eliminación de modelos y datos intermedios, así como la adición de nuevas matrices de adyacencia para pensiones.
</commit_message>
<xml_diff>
--- a/Modelo/datos/Intermedias/Casos.xlsx
+++ b/Modelo/datos/Intermedias/Casos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/21a7d57e8591b932/Escritorio/CICS/2025/Tesis/Objetivos de Aprendizaje/Modelo/datos/Intermedias/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="131" documentId="8_{E8B120D2-53B5-471F-9AEE-969F764F6DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{334BA673-0242-4E78-98FA-A76E3EA16B83}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="8_{E8B120D2-53B5-471F-9AEE-969F764F6DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FCC8B9B-ECFF-4D0C-B7F7-70622AC86354}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -956,6 +956,12 @@
       <c r="D25">
         <v>1</v>
       </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26">
@@ -968,6 +974,12 @@
         <v>1</v>
       </c>
       <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
         <v>1</v>
       </c>
     </row>

</xml_diff>